<commit_message>
feat(F-NAR-008): 22 ATOM de plus (vague 2 suite)
Politesse et différences : histoires, pas des listes.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-03.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le livre de trains d'Aniss</t>
+          <t>Le train bleu d'Aniss</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>COL.ECO.002</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -841,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut un livre de trains à la bibliothèque, puis une poire au marché. Il dit bonjour, s'il te plaît, merci aux deux endroits.</t>
+          <t>Aniss veut le livre de trains sous la lampe jaune. Il dit bonjour, s'il te plaît, merci. Le crayon bleu dessine la locomotive.</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1189,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La pluie dessine des fils sur la vitre. Les parapluies gouttent dans un seau de zinc. Ça sent le papier mouillé et le bois. Une lampe pose un rond jaune sur une table. Le tapis est épais, un peu rêche sous les bottes. Les étagères montent tout droit, jusqu'au plafond. Les dos des livres sont verts, rouges, bruns. Une horloge fait tic-tac, tout au fond. Tu as vu la pluie, Aniss ? Oui, maman. Elle coule tout droit. On est au chaud, ici. Le foulard bleu de maman sèche près du radiateur. En ce moment, Aniss s'arrête près d'une étagère basse. Il cherche un livre de trains. Ses doigts glissent sur les couvertures lisses. Maman, je veux un train. On va le demander à la dame. On dit bonjour d'abord. La dame des livres est derrière un bureau de bois. Un tampon repose près d'une pile de cartes. Aniss s'avance, tout près de maman. Bonjour. Bonjour. La dame lève les yeux. Sa voix est douce, comme le papier. Aniss montre un livre rouge, avec une locomotive. Le livre de trains, s'il te plaît. Très bien, Aniss. La dame tend le livre. La couverture est lisse, un peu froide. Merci. Bravo. Tu as dit merci. Aniss ouvre une page. Un train bleu roule sur un pont. Le papier sent le neuf. Il est tout bleu, maman. Oui. Tu l'as bien demandé. Ils restent un moment sous la lampe jaune. La pluie continue, tout contre la vitre. Plus tard, le seau de zinc est plein de gouttes. Ils sortent. Les bottes font un petit bruit sur les dalles mouillées. Le marché est plus loin, sous une bâche claire. Ça sent les poires et la terre humide. Les caisses sont mouillées, luisantes. Tu te souviens des mots, Aniss ? Bonjour. S'il te plaît. Merci. Oui. On les dit aussi ici. Aniss voit le marchand de poires. Une poire jaune brille, encore ronde. Bonjour. Le marchand incline la tête. Une poire, s'il te plaît. Le marchand pose la poire dans un petit sac. Le sac est un peu rêche. Merci. Bravo, Aniss. Tu as fait du bon travail. Tu as dit les mots ici aussi. Comme à la bibliothèque. Comme à la bibliothèque. Aniss tient le livre sous le bras. Il tient le sac de l'autre main. La poire sent le sucré, tout près du nez.</t>
+          <t>Le radiateur cliquette tout bas. Un foulard bleu sèche dessus. Il est lourd d'eau de pluie. Une horloge pousse un tic. Puis un tac, tout au fond. Une lampe pose un rond jaune. Le tapis est épais sous les bottes. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Dehors, la pluie tape le zinc. Les parapluies gouttent dans un seau. Ça sent le papier et le bois. Les étagères montent jusqu'au plafond. Les dos des livres sont verts, rouges, bruns. En ce moment, Aniss cherche un livre. Ses doigts glissent sur les dos lisses. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Le tampon fait toc, toc. Aniss attend près du bois. Le livre rouge est sur le chariot. Juste derrière elle. Il est là. On attend un peu. Elle a les mains pleines. Le tampon se pose enfin. La dame lève les yeux. Aniss montre le livre rouge. Tu demandes, Aniss.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Malik entre à la bibliothèque avec maman. Les livres sentent le papier. Il voit la dame des livres. Malik dit : &lt;emphasis level="moderate"&gt;bonjour&lt;/emphasis&gt;. La dame sourit. Malik veut un livre de trains. Il dit : s'il te plaît. La dame tend le livre. Malik dit : merci. Il touche la couverture. Elle est lisse. Plus tard, ils vont au marché. Les étals sentent les fruits. Malik voit le marchand de poires. Il se souvient. Il dit : bonjour. Il dit : une poire, s'il te plaît. Le marchand donne la poire. Malik dit : merci. Maman sourit. Même leçon, autre lieu. On salue. On demande. On remercie.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le radiateur cliquette tout bas. Un foulard bleu sèche dessus. Il est lourd d'eau de pluie. Une horloge pousse un tic. Puis un tac, tout au fond. Une lampe pose un rond jaune. Le tapis est épais sous les bottes. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Dehors, la pluie tape le zinc. Les parapluies gouttent dans un seau. Ça sent le papier et le bois. Les étagères montent jusqu'au plafond. Les dos des livres sont verts, rouges, bruns. En ce moment, Aniss cherche un livre. Ses doigts glissent sur les dos lisses. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Le tampon fait toc, toc. Aniss attend près du bois. Le livre rouge est sur le chariot. Juste derrière elle. Il est là. On attend un peu. Elle a les mains pleines. Le tampon se pose enfin. La dame lève les yeux. Aniss montre le livre rouge. Tu demandes, Aniss.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1252,7 +1257,7 @@
         <v>0.96</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1324,77 +1329,45 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t xml:space="preserve">narrateur|La pluie dessine des fils sur la vitre.
-narrateur|Les parapluies gouttent dans un seau de zinc.
-narrateur|Ça sent le papier mouillé et le bois.
-narrateur|Une lampe pose un rond jaune sur une table.
-narrateur|Le tapis est épais, un peu rêche sous les bottes.
-narrateur|Les étagères montent tout droit, jusqu'au plafond.
+          <t>narrateur|Le radiateur cliquette tout bas.
+narrateur|Un foulard bleu sèche dessus.
+narrateur|Il est lourd d'eau de pluie.
+narrateur|Une horloge pousse un tic.
+narrateur|Puis un tac, tout au fond.
+narrateur|Une lampe pose un rond jaune.
+narrateur|Le tapis est épais sous les bottes.
+maman|Tu entends l'horloge, Aniss ?
+enfant-m|Tic.
+enfant-m|Tac.
+papa|On est au chaud, ici.
+narrateur|Dehors, la pluie tape le zinc.
+narrateur|Les parapluies gouttent dans un seau.
+narrateur|Ça sent le papier et le bois.
+narrateur|Les étagères montent jusqu'au plafond.
 narrateur|Les dos des livres sont verts, rouges, bruns.
-narrateur|Une horloge fait tic-tac, tout au fond.
-maman|Tu as vu la pluie, Aniss ?
-enfant-m|Oui, maman.
-enfant-m|Elle coule tout droit.
-maman|On est au chaud, ici.
-narrateur|Le foulard bleu de maman sèche près du radiateur.
-narrateur|En ce moment, Aniss s'arrête près d'une étagère basse.
-narrateur|Il cherche un livre de trains.
-narrateur|Ses doigts glissent sur les couvertures lisses.
-enfant-m|Maman, je veux un train.
-maman|On va le demander à la dame.
-maman|On dit bonjour d'abord.
-narrateur|La dame des livres est derrière un bureau de bois.
-narrateur|Un tampon repose près d'une pile de cartes.
-narrateur|Aniss s'avance, tout près de maman.
-enfant-m|Bonjour.
-maman|Bonjour.
+narrateur|En ce moment, Aniss cherche un livre.
+narrateur|Ses doigts glissent sur les dos lisses.
+enfant-m|Maman, un train.
+enfant-m|Il est rouge.
+maman|Celui avec la locomotive.
+papa|On s'approche du bureau.
+narrateur|La dame tamponne des cartes.
+narrateur|Le tampon fait toc, toc.
+narrateur|Aniss attend près du bois.
+narrateur|Le livre rouge est sur le chariot.
+narrateur|Juste derrière elle.
+enfant-m|Il est là.
+maman|On attend un peu.
+papa|Elle a les mains pleines.
+narrateur|Le tampon se pose enfin.
 narrateur|La dame lève les yeux.
-narrateur|Sa voix est douce, comme le papier.
-narrateur|Aniss montre un livre rouge, avec une locomotive.
-enfant-m|Le livre de trains, s'il te plaît.
-maman|Très bien, Aniss.
-narrateur|La dame tend le livre.
-narrateur|La couverture est lisse, un peu froide.
-enfant-m|Merci.
-maman|Bravo.
-maman|Tu as dit merci.
-narrateur|Aniss ouvre une page.
-narrateur|Un train bleu roule sur un pont.
-narrateur|Le papier sent le neuf.
-enfant-m|Il est tout bleu, maman.
-maman|Oui.
-maman|Tu l'as bien demandé.
-narrateur|Ils restent un moment sous la lampe jaune.
-narrateur|La pluie continue, tout contre la vitre.
-narrateur|Plus tard, le seau de zinc est plein de gouttes.
-narrateur|Ils sortent.
-narrateur|Les bottes font un petit bruit sur les dalles mouillées.
-narrateur|Le marché est plus loin, sous une bâche claire.
-narrateur|Ça sent les poires et la terre humide.
-narrateur|Les caisses sont mouillées, luisantes.
-maman|Tu te souviens des mots, Aniss ?
-enfant-m|Bonjour.
-enfant-m|S'il te plaît.
-enfant-m|Merci.
-maman|Oui.
-maman|On les dit aussi ici.
-narrateur|Aniss voit le marchand de poires.
-narrateur|Une poire jaune brille, encore ronde.
-enfant-m|Bonjour.
-narrateur|Le marchand incline la tête.
-enfant-m|Une poire, s'il te plaît.
-narrateur|Le marchand pose la poire dans un petit sac.
-narrateur|Le sac est un peu rêche.
-enfant-m|Merci.
-maman|Bravo, Aniss.
-maman|Tu as fait du bon travail.
-maman|Tu as dit les mots ici aussi.
-enfant-m|Comme à la bibliothèque.
-maman|Comme à la bibliothèque.
-narrateur|Aniss tient le livre sous le bras.
-narrateur|Il tient le sac de l'autre main.
-narrateur|La poire sent le sucré, tout près du nez.
-</t>
+narrateur|Aniss montre le livre rouge.
+maman|Tu demandes, Aniss.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>horloge,pluie</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1394,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Aniss parle à la dame. Quels mots dit-il ?</t>
+          <t>Aniss veut le livre. Que dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Malik parle à la dame. Quels mots dit-il ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Aniss veut le livre. Que dit-il ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1456,7 +1429,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit bonjour. Il dit s'il te plaît. Il dit merci. Quels mots ?</t>
+          <t>Il dit bonjour. Que dit Aniss ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1577,9 +1550,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t xml:space="preserve">narrateur|Aniss parle à la dame.
-narrateur|Quels mots dit-il ?
-</t>
+          <t>narrateur|Aniss veut le livre.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1606,12 +1578,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss serre le livre contre son manteau. La couverture reste lisse sous sa main. Quels mots tu as dits, Aniss ? Bonjour. S'il te plaît. Merci. Oui. À la bibliothèque. Et au marché aussi. Bravo. C'est du bon travail. La poire roule un peu dans le sac. Aniss l'entend, tout doux. Elle est jaune, maman. Oui. Tu l'as demandée. Tu as dit s'il te plaît.</t>
+          <t>Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Plus tard, le seau de zinc est plein. Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Une petite boutique a des crayons. Un crayon bleu brille dans un pot. Pour le train. Bonjour. Un crayon bleu, s'il te plaît. La dame du pot tend le crayon. Le bois est lisse, un peu sec. Merci. On rentre, maintenant. Aniss tient le livre. Il tient le crayon, tout droit.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Malik a dit &lt;emphasis level="moderate"&gt;bonjour&lt;/emphasis&gt;. Puis s'il te plaît. Puis merci. À la bibliothèque, puis au marché.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Plus tard, le seau de zinc est plein. Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Une petite boutique a des crayons. Un crayon bleu brille dans un pot. Pour le train. Bonjour. Un crayon bleu, s'il te plaît. La dame du pot tend le crayon. Le bois est lisse, un peu sec. Merci. On rentre, maintenant. Aniss tient le livre. Il tient le crayon, tout droit.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1674,7 +1646,7 @@
         <v>0.96</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1750,24 +1722,40 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t xml:space="preserve">narrateur|Aniss serre le livre contre son manteau.
-narrateur|La couverture reste lisse sous sa main.
-maman|Quels mots tu as dits, Aniss ?
+          <t>enfant-m|Bonjour.
+maman|Bonjour.
+enfant-m|Le livre de trains, s'il te plaît.
+enfant-m|Celui avec la locomotive.
+narrateur|La dame tend le livre rouge.
+narrateur|La couverture est lisse, un peu froide.
+enfant-m|Merci.
+papa|Merci.
+narrateur|Aniss ouvre une page.
+narrateur|Un train bleu roule sur un pont.
+enfant-m|Il est tout bleu, papa.
+papa|Oui.
+maman|Tu l'as dans les mains.
+narrateur|Ils restent sous la lampe jaune.
+narrateur|La pluie continue contre la vitre.
+narrateur|Plus tard, le seau de zinc est plein.
+narrateur|Ils sortent, le livre sous le bras.
+narrateur|Les bottes sonnent sur les dalles mouillées.
+narrateur|Une petite boutique a des crayons.
+narrateur|Un crayon bleu brille dans un pot.
+enfant-m|Pour le train.
 enfant-m|Bonjour.
-enfant-m|S'il te plaît.
+enfant-m|Un crayon bleu, s'il te plaît.
+narrateur|La dame du pot tend le crayon.
+narrateur|Le bois est lisse, un peu sec.
 enfant-m|Merci.
-maman|Oui.
-maman|À la bibliothèque.
-maman|Et au marché aussi.
-maman|Bravo.
-maman|C'est du bon travail.
-narrateur|La poire roule un peu dans le sac.
-narrateur|Aniss l'entend, tout doux.
-enfant-m|Elle est jaune, maman.
-maman|Oui.
-maman|Tu l'as demandée.
-maman|Tu as dit s'il te plaît.
-</t>
+maman|On rentre, maintenant.
+narrateur|Aniss tient le livre.
+narrateur|Il tient le crayon, tout droit.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>papier,pas</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1782,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent sous un parapluie partagé. Les gouttes tapent le tissu, une par une. À la maison, maman pose le livre sur la table. Aniss pose la poire dans une assiette. Tu veux un bout de poire ? Oui, maman. La poire est juteuse, un peu froide. Merci, maman. Merci, Aniss. On a eu le livre. On a eu la poire. On a dit les mots. Bonjour, s'il te plaît, merci. Bravo. Le train bleu attend sur la page. La pluie finit, tout loin.</t>
+          <t>À la maison, le foulard est presque sec. Aniss pose le livre sur la table. Il ouvre la page du pont. Tu veux le crayon ? Oui, maman. S'il te plaît. Le crayon bleu glisse sur le papier. Une locomotive apparaît, tout simple. C'est mon train. Il a un pont, comme le livre. Oui. Il est bleu, hein ? Tout bleu. La pluie est plus douce, dehors. Tu tiens le livre des deux mains ? Oui, papa. Le crayon sent un peu le bois. La page reste ouverte, près de lui. On le laisse ouvert ? Oui. Le pont est encore là.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Malik tient le livre et la poire. Maman dit &lt;emphasis level="moderate"&gt;merci&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>À la maison, le foulard est presque sec. Aniss pose le livre sur la table. Il ouvre la page du pont. Tu veux le crayon ? Oui, maman. S'il te plaît. Le crayon bleu glisse sur le papier. Une locomotive apparaît, tout simple. C'est mon train. Il a un pont, comme le livre. Oui. Il est bleu, hein ? Tout bleu. La pluie est plus douce, dehors. Tu tiens le livre des deux mains ? Oui, papa. Le crayon sent un peu le bois. La page reste ouverte, près de lui. On le laisse ouvert ? Oui. Le pont est encore là.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1862,7 +1850,7 @@
         <v>0.96</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1934,23 +1922,32 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t xml:space="preserve">narrateur|Ils rentrent sous un parapluie partagé.
-narrateur|Les gouttes tapent le tissu, une par une.
-narrateur|À la maison, maman pose le livre sur la table.
-narrateur|Aniss pose la poire dans une assiette.
-maman|Tu veux un bout de poire ?
+          <t>narrateur|À la maison, le foulard est presque sec.
+narrateur|Aniss pose le livre sur la table.
+narrateur|Il ouvre la page du pont.
+maman|Tu veux le crayon ?
 enfant-m|Oui, maman.
-narrateur|La poire est juteuse, un peu froide.
-enfant-m|Merci, maman.
-maman|Merci, Aniss.
-maman|On a eu le livre.
-maman|On a eu la poire.
-maman|On a dit les mots.
-enfant-m|Bonjour, s'il te plaît, merci.
-maman|Bravo.
-narrateur|Le train bleu attend sur la page.
-narrateur|La pluie finit, tout loin.
-</t>
+enfant-m|S'il te plaît.
+narrateur|Le crayon bleu glisse sur le papier.
+narrateur|Une locomotive apparaît, tout simple.
+enfant-m|C'est mon train.
+papa|Il a un pont, comme le livre.
+enfant-m|Oui.
+maman|Il est bleu, hein ?
+enfant-m|Tout bleu.
+narrateur|La pluie est plus douce, dehors.
+papa|Tu tiens le livre des deux mains ?
+enfant-m|Oui, papa.
+narrateur|Le crayon sent un peu le bois.
+narrateur|La page reste ouverte, près de lui.
+maman|On le laisse ouvert ?
+enfant-m|Oui.
+papa|Le pont est encore là.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>crayon</t>
         </is>
       </c>
     </row>
@@ -1977,12 +1974,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit bonjour. J'ai dit s'il te plaît. J'ai dit merci. Bravo, Aniss. Tu as fait du bon travail. L'histoire est finie.</t>
+          <t>Le crayon repose près du livre. Le train bleu est sur le papier. Bonne soirée, Aniss. Il a un pont, ton train. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le crayon repose près du livre. Le train bleu est sur le papier. Bonne soirée, Aniss. Il a un pont, ton train. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2117,13 +2114,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t xml:space="preserve">enfant-m|J'ai dit bonjour.
-enfant-m|J'ai dit s'il te plaît.
-enfant-m|J'ai dit merci.
-maman|Bravo, Aniss.
-maman|Tu as fait du bon travail.
-narrateur|L'histoire est finie.
-</t>
+          <t>narrateur|Le crayon repose près du livre.
+narrateur|Le train bleu est sur le papier.
+maman|Bonne soirée, Aniss.
+papa|Il a un pont, ton train.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2219,13 @@
       <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-03 Le livre de trains d'Aniss
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-03.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le train bleu d'Aniss</t>
+          <t>Le livre de trains d'Aniss</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bibliothèque sous la pluie, puis boutique de crayons</t>
+          <t>bibliothèque puis marché</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut le livre de trains sous la lampe jaune. Il dit bonjour, s'il te plaît, merci. Le crayon bleu dessine la locomotive.</t>
+          <t>Une goutte court sur le tissu sombre. Sur le parapluie fermé, un éclat de parapluie brille. Aniss veut le livre de trains, maintenant. Il parle trop vite : les mots se cognent au tampon. La dame ne lève pas les yeux. Sourire parti. Papa se baisse. Bonjour, s'il te plaît, merci vécus. Au marché, le papier mouillé glisse. Il refuse de foncer. Sur le tissu, l'éclat de parapluie tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur cliquette tout bas. Un foulard bleu sèche dessus. Il est lourd d'eau de pluie. Une horloge pousse un tic. Puis un tac, tout au fond. Une lampe pose un rond jaune. Le tapis est épais sous les bottes. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Dehors, la pluie tape le zinc. Les parapluies gouttent dans un seau. Ça sent le papier et le bois. Les étagères montent jusqu'au plafond. Les dos des livres sont verts, rouges, bruns. En ce moment, Aniss cherche un livre. Ses doigts glissent sur les dos lisses. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Le tampon fait toc, toc. Aniss attend près du bois. Le livre rouge est sur le chariot. Juste derrière elle. Il est là. On attend un peu. Elle a les mains pleines. Le tampon se pose enfin. La dame lève les yeux. Aniss montre le livre rouge. Tu demandes, Aniss.</t>
+          <t>Une goutte court sur le tissu sombre. Un parapluie fermé penche vers le zinc. Les parapluies gouttent dans un seau de zinc. Ça sent le papier mouillé et le bois. Une lampe pose un rond jaune sur une table. Le tapis est épais, un peu rêche sous les bottes. Les étagères montent jusqu'au plafond. Sur le tissu, un éclat de parapluie brille. Il brille, papa. C'est l'eau, sous la lumière. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le foulard bleu sèche près du radiateur. Le foulard est lourd d'eau de pluie. Je veux un livre de trains ! Celui avec la locomotive ? Oui, tout de suite ! En ce moment, Aniss s'arrête près d'une étagère basse. Ses doigts glissent sur les couvertures lisses. Les dos des livres sont verts, rouges, bruns. Une horloge pousse un tic, au fond. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Un tampon repose près d'une pile de cartes. Le tampon fait toc, toc. Le livre rouge est sur le chariot. Juste derrière le bureau de bois. Le train ! Les mots d'Aniss se cognent au tampon. La dame ne lève pas les yeux. Ses mains sont pleines de cartes. Oh. L'éclat de parapluie tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Elle ne me voit pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le livre est derrière le bois ? Oui, papa. Aniss montre le livre rouge, avec une locomotive. Tu parles à la dame, Aniss. Le tampon se pose enfin. La dame lève les yeux. Il est là. Elle te regarde, Aniss ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le radiateur cliquette tout bas. Un foulard bleu sèche dessus. Il est lourd d'eau de pluie. Une horloge pousse un tic. Puis un tac, tout au fond. Une lampe pose un rond jaune. Le tapis est épais sous les bottes. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Dehors, la pluie tape le zinc. Les parapluies gouttent dans un seau. Ça sent le papier et le bois. Les étagères montent jusqu'au plafond. Les dos des livres sont verts, rouges, bruns. En ce moment, Aniss cherche un livre. Ses doigts glissent sur les dos lisses. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Le tampon fait toc, toc. Aniss attend près du bois. Le livre rouge est sur le chariot. Juste derrière elle. Il est là. On attend un peu. Elle a les mains pleines. Le tampon se pose enfin. La dame lève les yeux. Aniss montre le livre rouge. Tu demandes, Aniss.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte court sur le tissu sombre. Un parapluie fermé penche vers le zinc. Les parapluies gouttent dans un seau de zinc. Ça sent le papier mouillé et le bois. Une lampe pose un rond jaune sur une table. Le tapis est épais, un peu rêche sous les bottes. Les étagères montent jusqu'au plafond. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de parapluie&lt;/emphasis&gt; brille. Il brille, papa. C'est l'eau, sous la lumière. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le foulard bleu sèche près du radiateur. Le foulard est lourd d'eau de pluie. Je veux un livre de trains ! Celui avec la locomotive ? Oui, tout de suite ! En ce moment, Aniss s'arrête près d'une étagère basse. Ses doigts glissent sur les couvertures lisses. Les dos des livres sont verts, rouges, bruns. Une horloge pousse un tic, au fond. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Un tampon repose près d'une pile de cartes. Le tampon fait toc, toc. Le livre rouge est sur le chariot. Juste derrière le bureau de bois. Le train ! Les mots d'Aniss se cognent au tampon. La dame ne lève pas les yeux. Ses mains sont pleines de cartes. Oh. L'éclat de parapluie tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Elle ne me voit pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le livre est derrière le bois ? Oui, papa. Aniss montre le livre rouge, avec une locomotive. Tu parles à la dame, Aniss. Le tampon se pose enfin. La dame lève les yeux. Il est là. Elle te regarde, Aniss ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Malik entre à la bibliothèque avec maman. Les livres sentent le papier. Il voit la dame des livres. Malik dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. La dame sourit. Malik veut un livre de trains. Il dit : s'il te plaît. La dame tend le livre. Malik dit : merci. Il touche la couverture. Elle est lisse. Plus tard, ils vont au marché. Les étals sentent les fruits. Malik voit le marchand de poires. Il se souvient. Il dit : bonjour. Il dit : une poire, s'il te plaît. Le marchand donne la poire. Malik dit : merci. Maman sourit. Même leçon, autre lieu. On salue. On demande. On remercie. [pause]</t>
+          <t>Une goutte court sur le tissu sombre. Un parapluie fermé penche vers le zinc. Les parapluies gouttent dans un seau de zinc. Ça sent le papier mouillé et le bois. Une lampe pose un rond jaune sur une table. Le tapis est épais, un peu rêche sous les bottes. Les étagères montent jusqu'au plafond. Sur le tissu, un &lt;emphasis&gt;éclat de parapluie&lt;/emphasis&gt; brille. Il brille, papa. C'est l'eau, sous la lumière. Papa tient la main d'Aniss. Ta main est bien dans la mienne. Le foulard bleu sèche près du radiateur. Le foulard est lourd d'eau de pluie. Je veux un livre de trains ! Celui avec la locomotive ? Oui, tout de suite ! En ce moment, Aniss s'arrête près d'une étagère basse. Ses doigts glissent sur les couvertures lisses. Les dos des livres sont verts, rouges, bruns. Une horloge pousse un tic, au fond. Tu entends l'horloge, Aniss ? Tic. Tac. On est au chaud, ici. Maman, un train. Il est rouge. Celui avec la locomotive. On s'approche du bureau. La dame tamponne des cartes. Un tampon repose près d'une pile de cartes. Le tampon fait toc, toc. Le livre rouge est sur le chariot. Juste derrière le bureau de bois. Le train ! Les mots d'Aniss se cognent au tampon. La dame ne lève pas les yeux. Ses mains sont pleines de cartes. Oh. L'éclat de parapluie tremble, puis tient. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Elle ne me voit pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Le livre est derrière le bois ? Oui, papa. Aniss montre le livre rouge, avec une locomotive. Tu parles à la dame, Aniss. Le tampon se pose enfin. La dame lève les yeux. Il est là. Elle te regarde, Aniss ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de parapluie</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,48 +1326,72 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_livre_de_trains_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le radiateur cliquette tout bas.
-narrateur|Un foulard bleu sèche dessus.
-narrateur|Il est lourd d'eau de pluie.
-narrateur|Une horloge pousse un tic.
-narrateur|Puis un tac, tout au fond.
-narrateur|Une lampe pose un rond jaune.
-narrateur|Le tapis est épais sous les bottes.
-maman|Tu entends l'horloge, Aniss ?
+          <t>narrateur|Une goutte court sur le tissu sombre.
+narrateur|Un parapluie fermé penche vers le zinc.
+narrateur|Les parapluies gouttent dans un seau de zinc.
+narrateur|Ça sent le papier mouillé et le bois.
+narrateur|Une lampe pose un rond jaune sur une table.
+narrateur|Le tapis est épais, un peu rêche sous les bottes.
+narrateur|Les étagères montent jusqu'au plafond.
+narrateur|Sur le tissu, un éclat de parapluie brille.
+enfant-m|Il brille, papa.
+papa|C'est l'eau, sous la lumière.
+narrateur|Papa tient la main d'Aniss.
+papa|Ta main est bien dans la mienne.
+maman|Le foulard bleu sèche près du radiateur.
+narrateur|Le foulard est lourd d'eau de pluie.
+enfant-m|Je veux un livre de trains !
+maman|Celui avec la locomotive ?
+enfant-m|Oui, tout de suite !
+narrateur|En ce moment, Aniss s'arrête près d'une étagère basse.
+narrateur|Ses doigts glissent sur les couvertures lisses.
+narrateur|Les dos des livres sont verts, rouges, bruns.
+narrateur|Une horloge pousse un tic, au fond.
+papa|Tu entends l'horloge, Aniss ?
 enfant-m|Tic.
 enfant-m|Tac.
-papa|On est au chaud, ici.
-narrateur|Dehors, la pluie tape le zinc.
-narrateur|Les parapluies gouttent dans un seau.
-narrateur|Ça sent le papier et le bois.
-narrateur|Les étagères montent jusqu'au plafond.
-narrateur|Les dos des livres sont verts, rouges, bruns.
-narrateur|En ce moment, Aniss cherche un livre.
-narrateur|Ses doigts glissent sur les dos lisses.
+maman|On est au chaud, ici.
 enfant-m|Maman, un train.
 enfant-m|Il est rouge.
 maman|Celui avec la locomotive.
 papa|On s'approche du bureau.
 narrateur|La dame tamponne des cartes.
+narrateur|Un tampon repose près d'une pile de cartes.
 narrateur|Le tampon fait toc, toc.
-narrateur|Aniss attend près du bois.
 narrateur|Le livre rouge est sur le chariot.
-narrateur|Juste derrière elle.
-enfant-m|Il est là.
-maman|On attend un peu.
-papa|Elle a les mains pleines.
+narrateur|Juste derrière le bureau de bois.
+enfant-m|Le train !
+narrateur|Les mots d'Aniss se cognent au tampon.
+narrateur|La dame ne lève pas les yeux.
+narrateur|Ses mains sont pleines de cartes.
+enfant-m|Oh.
+narrateur|L'éclat de parapluie tremble, puis tient.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+enfant-m|Elle ne me voit pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Le livre est derrière le bois ?
+enfant-m|Oui, papa.
+narrateur|Aniss montre le livre rouge, avec une locomotive.
+maman|Tu parles à la dame, Aniss.
 narrateur|Le tampon se pose enfin.
 narrateur|La dame lève les yeux.
-narrateur|Aniss montre le livre rouge.
-maman|Tu demandes, Aniss.</t>
+enfant-m|Il est là.
+papa|Elle te regarde, Aniss ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>horloge,pluie</t>
+          <t>pluie,parapluie</t>
         </is>
       </c>
     </row>
@@ -1394,17 +1418,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Aniss veut le livre. Que dit-il ?</t>
+          <t>Aniss parle à la dame. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss veut le livre. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Malik parle à la dame. Quels mots dit-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1429,7 +1453,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit bonjour. Que dit Aniss ?</t>
+          <t>Il dit bonjour. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1467,18 +1491,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,34 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1529,29 +1557,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_parle_a_la_dame_avec_bonjour; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Aniss veut le livre.
-narrateur|Que dit-il ?</t>
+          <t>narrateur|Aniss parle à la dame.
+narrateur|Quels mots dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1578,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Plus tard, le seau de zinc est plein. Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Une petite boutique a des crayons. Un crayon bleu brille dans un pot. Pour le train. Bonjour. Un crayon bleu, s'il te plaît. La dame du pot tend le crayon. Le bois est lisse, un peu sec. Merci. On rentre, maintenant. Aniss tient le livre. Il tient le crayon, tout droit.</t>
+          <t>Le train. Aniss referme la bouche. Aniss refuse de foncer. Personne ne parle. Il observe le tampon, un instant. Il écoute le silence du bureau. Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci, Aniss. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Aniss tourne une page, sans se presser. Le pont est petit. Il tient au-dessus de l'eau. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Le papier sent le neuf. Il roule sur le pont. On le voit bien. Aniss serre le livre contre son manteau. Le foulard est près de la porte. On sort, maman ? Oui, avec le livre. Le seau de zinc est plein de gouttes.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Plus tard, le seau de zinc est plein. Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Une petite boutique a des crayons. Un crayon bleu brille dans un pot. Pour le train. Bonjour. Un crayon bleu, s'il te plaît. La dame du pot tend le crayon. Le bois est lisse, un peu sec. Merci. On rentre, maintenant. Aniss tient le livre. Il tient le crayon, tout droit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le train. Aniss referme la bouche. Aniss refuse de foncer. Personne ne parle. Il observe le tampon, un instant. Il écoute le silence du bureau. Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci, Aniss. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Aniss tourne une page, sans se presser. Le pont est petit. Il tient au-dessus de l'eau. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Le papier sent le neuf. Il roule sur le pont. On le voit bien. Aniss serre le livre contre son manteau. Le foulard est près de la porte. On sort, maman ? Oui, avec le livre. Le seau de zinc est plein de gouttes.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Malik a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Puis s'il te plaît. Puis merci. À la bibliothèque, puis au marché. [pause]</t>
+          <t>Le train. Aniss referme la bouche. Aniss refuse de foncer. Personne ne parle. Il observe le tampon, un instant. Il écoute le silence du bureau. Bonjour. Bonjour. Le livre de trains, s'il te plaît. Celui avec la locomotive. La dame tend le livre rouge. La couverture est lisse, un peu froide. Merci. Merci, Aniss. Aniss ouvre une page. Un train bleu roule sur un pont. Il est tout bleu, papa. Oui. Aniss tourne une page, sans se presser. Le pont est petit. Il tient au-dessus de l'eau. Tu l'as dans les mains. Ils restent sous la lampe jaune. La pluie continue contre la vitre. Le papier sent le neuf. Il roule sur le pont. On le voit bien. Aniss serre le livre contre son manteau. Le foulard est près de la porte. On sort, maman ? Oui, avec le livre. Le seau de zinc est plein de gouttes. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1635,7 +1663,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1643,10 +1671,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1676,23 +1704,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1701,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1717,45 +1745,48 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bonjour_s_il_te_plait_merci_vecus; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
-maman|Bonjour.
+          <t>enfant-m|Le train.
+narrateur|Aniss referme la bouche.
+narrateur|Aniss refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe le tampon, un instant.
+narrateur|Il écoute le silence du bureau.
+enfant-m|Bonjour.
+papa|Bonjour.
 enfant-m|Le livre de trains, s'il te plaît.
 enfant-m|Celui avec la locomotive.
 narrateur|La dame tend le livre rouge.
 narrateur|La couverture est lisse, un peu froide.
 enfant-m|Merci.
-papa|Merci.
+papa|Merci, Aniss.
 narrateur|Aniss ouvre une page.
 narrateur|Un train bleu roule sur un pont.
 enfant-m|Il est tout bleu, papa.
 papa|Oui.
+narrateur|Aniss tourne une page, sans se presser.
+enfant-m|Le pont est petit.
+papa|Il tient au-dessus de l'eau.
 maman|Tu l'as dans les mains.
 narrateur|Ils restent sous la lampe jaune.
 narrateur|La pluie continue contre la vitre.
-narrateur|Plus tard, le seau de zinc est plein.
-narrateur|Ils sortent, le livre sous le bras.
-narrateur|Les bottes sonnent sur les dalles mouillées.
-narrateur|Une petite boutique a des crayons.
-narrateur|Un crayon bleu brille dans un pot.
-enfant-m|Pour le train.
-enfant-m|Bonjour.
-enfant-m|Un crayon bleu, s'il te plaît.
-narrateur|La dame du pot tend le crayon.
-narrateur|Le bois est lisse, un peu sec.
-enfant-m|Merci.
-maman|On rentre, maintenant.
-narrateur|Aniss tient le livre.
-narrateur|Il tient le crayon, tout droit.</t>
+narrateur|Le papier sent le neuf.
+enfant-m|Il roule sur le pont.
+maman|On le voit bien.
+narrateur|Aniss serre le livre contre son manteau.
+papa|Le foulard est près de la porte.
+enfant-m|On sort, maman ?
+maman|Oui, avec le livre.
+narrateur|Le seau de zinc est plein de gouttes.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>papier,pas</t>
+          <t>papier,livre</t>
         </is>
       </c>
     </row>
@@ -1782,17 +1813,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>À la maison, le foulard est presque sec. Aniss pose le livre sur la table. Il ouvre la page du pont. Tu veux le crayon ? Oui, maman. S'il te plaît. Le crayon bleu glisse sur le papier. Une locomotive apparaît, tout simple. C'est mon train. Il a un pont, comme le livre. Oui. Il est bleu, hein ? Tout bleu. La pluie est plus douce, dehors. Tu tiens le livre des deux mains ? Oui, papa. Le crayon sent un peu le bois. La page reste ouverte, près de lui. On le laisse ouvert ? Oui. Le pont est encore là.</t>
+          <t>Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Le marché est plus loin, sous une bâche claire. Ça sent les poires et la terre humide. Les caisses sont mouillées, luisantes. Une poire jaune ! Celle-là, bien ronde ? Oui, maman. Aniss tend la main trop vite. Le papier mouillé glisse sous ses doigts. La poire penche, puis retombe. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Aniss refuse de foncer. Personne ne parle. Il observe la caisse, un instant. Il écoute la pluie sur la bâche. Sur le parapluie de papa, l'éclat de parapluie brille. Bonjour. Le marchand incline la tête. Une poire, s'il te plaît. Le marchand pose la poire dans un petit sac. Le sac est un peu rêche. Merci. On rentre, maintenant. Tu tiens le livre des deux mains ? Oui, papa. Aniss tient le livre sous le bras. Il tient le sac de l'autre main. La poire sent le sucré, près du nez.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>À la maison, le foulard est presque sec. Aniss pose le livre sur la table. Il ouvre la page du pont. Tu veux le crayon ? Oui, maman. S'il te plaît. Le crayon bleu glisse sur le papier. Une locomotive apparaît, tout simple. C'est mon train. Il a un pont, comme le livre. Oui. Il est bleu, hein ? Tout bleu. La pluie est plus douce, dehors. Tu tiens le livre des deux mains ? Oui, papa. Le crayon sent un peu le bois. La page reste ouverte, près de lui. On le laisse ouvert ? Oui. Le pont est encore là.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Le marché est plus loin, sous une bâche claire. Ça sent les poires et la terre humide. Les caisses sont mouillées, luisantes. Une poire jaune ! Celle-là, bien ronde ? Oui, maman. Aniss tend la main trop vite. Le &lt;emphasis level="moderate"&gt;papier mouillé&lt;/emphasis&gt; glisse sous ses doigts. La poire penche, puis retombe. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Aniss refuse de foncer. Personne ne parle. Il observe la caisse, un instant. Il écoute la pluie sur la bâche. Sur le parapluie de papa, l'éclat de parapluie brille. Bonjour. Le marchand incline la tête. Une poire, s'il te plaît. Le marchand pose la poire dans un petit sac. Le sac est un peu rêche. Merci. On rentre, maintenant. Tu tiens le livre des deux mains ? Oui, papa. Aniss tient le livre sous le bras. Il tient le sac de l'autre main. La poire sent le sucré, près du nez.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Malik tient le livre et la poire. Maman dit &lt;emphasis&gt;merci&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils sortent, le livre sous le bras. Les bottes sonnent sur les dalles mouillées. Le marché est plus loin, sous une bâche claire. Ça sent les poires et la terre humide. Les caisses sont mouillées, luisantes. Une poire jaune ! Celle-là, bien ronde ? Oui, maman. Aniss tend la main trop vite. Le &lt;emphasis&gt;papier mouillé&lt;/emphasis&gt; glisse sous ses doigts. La poire penche, puis retombe. Oh. Aniss s'arrête. Ses mains se ferment, puis s'ouvrent. Aniss refuse de foncer. Personne ne parle. Il observe la caisse, un instant. Il écoute la pluie sur la bâche. Sur le parapluie de papa, l'éclat de parapluie brille. Bonjour. Le marchand incline la tête. Une poire, s'il te plaît. Le marchand pose la poire dans un petit sac. Le sac est un peu rêche. Merci. On rentre, maintenant. Tu tiens le livre des deux mains ? Oui, papa. Aniss tient le livre sous le bras. Il tient le sac de l'autre main. La poire sent le sucré, près du nez. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1839,7 +1870,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1847,10 +1878,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1873,30 +1904,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>merci</t>
+          <t>papier mouillé</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1905,10 +1936,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1919,35 +1950,49 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_la_poire; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|À la maison, le foulard est presque sec.
-narrateur|Aniss pose le livre sur la table.
-narrateur|Il ouvre la page du pont.
-maman|Tu veux le crayon ?
+          <t>narrateur|Ils sortent, le livre sous le bras.
+narrateur|Les bottes sonnent sur les dalles mouillées.
+narrateur|Le marché est plus loin, sous une bâche claire.
+narrateur|Ça sent les poires et la terre humide.
+narrateur|Les caisses sont mouillées, luisantes.
+enfant-m|Une poire jaune !
+maman|Celle-là, bien ronde ?
 enfant-m|Oui, maman.
-enfant-m|S'il te plaît.
-narrateur|Le crayon bleu glisse sur le papier.
-narrateur|Une locomotive apparaît, tout simple.
-enfant-m|C'est mon train.
-papa|Il a un pont, comme le livre.
-enfant-m|Oui.
-maman|Il est bleu, hein ?
-enfant-m|Tout bleu.
-narrateur|La pluie est plus douce, dehors.
+narrateur|Aniss tend la main trop vite.
+narrateur|Le papier mouillé glisse sous ses doigts.
+narrateur|La poire penche, puis retombe.
+enfant-m|Oh.
+narrateur|Aniss s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Aniss refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe la caisse, un instant.
+narrateur|Il écoute la pluie sur la bâche.
+narrateur|Sur le parapluie de papa, l'éclat de parapluie brille.
+enfant-m|Bonjour.
+narrateur|Le marchand incline la tête.
+enfant-m|Une poire, s'il te plaît.
+narrateur|Le marchand pose la poire dans un petit sac.
+narrateur|Le sac est un peu rêche.
+enfant-m|Merci.
+maman|On rentre, maintenant.
 papa|Tu tiens le livre des deux mains ?
 enfant-m|Oui, papa.
-narrateur|Le crayon sent un peu le bois.
-narrateur|La page reste ouverte, près de lui.
-maman|On le laisse ouvert ?
-enfant-m|Oui.
-papa|Le pont est encore là.</t>
+narrateur|Aniss tient le livre sous le bras.
+narrateur|Il tient le sac de l'autre main.
+narrateur|La poire sent le sucré, près du nez.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>crayon</t>
+          <t>poire,marche</t>
         </is>
       </c>
     </row>
@@ -1974,17 +2019,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le crayon repose près du livre. Le train bleu est sur le papier. Bonne soirée, Aniss. Il a un pont, ton train.</t>
+          <t>Ils rentrent sous un parapluie partagé. Les gouttes tapent le tissu, une par une. À la maison, maman pose le livre sur la table. Aniss pose la poire dans une assiette. Tu veux un bout de poire ? Oui, maman. La poire est juteuse, un peu froide. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le tissu. On est bien, ici. Aniss glisse le parapluie près de la porte. Le tissu repose contre le zinc. On le voit, maman. Tu le vois sur le tissu ? Oui, l'éclat. Le train bleu attend sur la page. La pluie finit, plus loin. L'éclat de parapluie tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le crayon repose près du livre. Le train bleu est sur le papier. Bonne soirée, Aniss. Il a un pont, ton train.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent sous un parapluie partagé. Les gouttes tapent le tissu, une par une. À la maison, maman pose le livre sur la table. Aniss pose la poire dans une assiette. Tu veux un bout de poire ? Oui, maman. La poire est juteuse, un peu froide. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le tissu. On est bien, ici. Aniss glisse le parapluie près de la porte. Le tissu repose contre le zinc. On le voit, maman. Tu le vois sur le tissu ? Oui, l'éclat. Le train bleu attend sur la page. La pluie finit, plus loin. L'&lt;emphasis level="moderate"&gt;éclat de parapluie&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent sous un parapluie partagé. Les gouttes tapent le tissu, une par une. À la maison, maman pose le livre sur la table. Aniss pose la poire dans une assiette. Tu veux un bout de poire ? Oui, maman. La poire est juteuse, un peu froide. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le tissu. On est bien, ici. Aniss glisse le parapluie près de la porte. Le tissu repose contre le zinc. On le voit, maman. Tu le vois sur le tissu ? Oui, l'éclat. Le train bleu attend sur la page. La pluie finit, plus loin. L'&lt;emphasis&gt;éclat de parapluie&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2031,18 +2076,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2051,12 +2096,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2065,17 +2110,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de parapluie</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2084,11 +2133,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2097,27 +2146,51 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le crayon repose près du livre.
-narrateur|Le train bleu est sur le papier.
-maman|Bonne soirée, Aniss.
-papa|Il a un pont, ton train.</t>
+          <t>narrateur|Ils rentrent sous un parapluie partagé.
+narrateur|Les gouttes tapent le tissu, une par une.
+narrateur|À la maison, maman pose le livre sur la table.
+narrateur|Aniss pose la poire dans une assiette.
+maman|Tu veux un bout de poire ?
+enfant-m|Oui, maman.
+narrateur|La poire est juteuse, un peu froide.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le tissu.
+maman|On est bien, ici.
+narrateur|Aniss glisse le parapluie près de la porte.
+narrateur|Le tissu repose contre le zinc.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le tissu ?
+enfant-m|Oui, l'éclat.
+narrateur|Le train bleu attend sur la page.
+narrateur|La pluie finit, plus loin.
+narrateur|L'éclat de parapluie tient sur le tissu.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>parapluie</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2230,6 +2303,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>